<commit_message>
fix(req3): execute physical tests on real fan, add 3 hardware edge cases and explanation
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C88E23-129D-4E67-B194-182DA8CC62D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8E575F-6CD3-4F89-A583-CA0B76FF6DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="123">
   <si>
     <t>TEST CASE REQUIREMENT 3</t>
   </si>
@@ -318,6 +318,72 @@
   </si>
   <si>
     <t>Quạt tiếp tục vận hành ở Level 2 ngay khi có điện lại, không chập cháy hay tóe lửa bất thường tại phích cắm.</t>
+  </si>
+  <si>
+    <t>Kiểm tra lực cần thiết để rút chốt kéo tuốc-năng khi đầu quạt đang ở điểm tận cùng hành trình xoay (góc tối đa bên trái hoặc phải).</t>
+  </si>
+  <si>
+    <t>Quạt đang bật tuốc-năng xoay Level 2; Chờ đầu quạt đến điểm tận cùng hành trình rồi kéo chốt lên ngay.</t>
+  </si>
+  <si>
+    <t>1. Bật quạt Level 2 và bật tuốc-năng.2. Quan sát đầu quạt xoay qua lại.3. Khi đầu quạt đạt góc tận cùng tối đa (trái hoặc phải), kéo chốt tuốc-năng lên ngay lập tức.4. So sánh lực kéo với lúc rút chốt ở vị trí giữa hành trình.</t>
+  </si>
+  <si>
+    <t>Chốt kéo lên nhẹ nhàng như bình thường bất kể đầu quạt đang ở vị trí nào trong hành trình xoay.</t>
+  </si>
+  <si>
+    <t>Chốt nặng tay hơn rõ rệt và phải dùng lực lớn hơn mới kéo lên được do bánh cam đang ở vị trí chịu tải cơ học tối đa tại điểm tận cùng hành trình.</t>
+  </si>
+  <si>
+    <t>FAIL (Chốt kẹt cứng / Bánh cam ở điểm tải cực đại)</t>
+  </si>
+  <si>
+    <t>Edge case AI bỏ sót</t>
+  </si>
+  <si>
+    <t>Kiểm tra phản hồi cơ học khi người dùng bấm lại đúng nút tốc độ đang gài để thử tắt quạt (bấm lại nút Level đang chạy).</t>
+  </si>
+  <si>
+    <t>Quạt đang chạy Level 2 (nút Level 2 đang gài xuống); Bấm đúng nút Level 2 thêm 1 lần nữa.</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy Level 2.2. Bấm nhấn lại nút Level 2 thêm 1 lần nữa.3. Quan sát xem quạt có tắt không.</t>
+  </si>
+  <si>
+    <t>Nút Level 2 nảy lên, quạt tắt đi (hành vi trực quan mà người dùng mong đợi).</t>
+  </si>
+  <si>
+    <t>Nút Level 2 không nảy lên, quạt vẫn tiếp tục chạy vì cơ chế nảy chỉ hoạt động khi một nút khác được bấm xuống, không có cơ chế tự nhả khi bấm lại cùng nút.</t>
+  </si>
+  <si>
+    <t>FAIL (Thiếu cơ chế tự nhả / gây nhầm lẫn UX)</t>
+  </si>
+  <si>
+    <t>Kiểm tra phản hồi cơ học khi bấm nút cấp tốc độ dở chừng (Half-press / Bấm nhẹ không hết hành trình).</t>
+  </si>
+  <si>
+    <t>Quạt đang chạy Level 1; Ấn nhẹ nút Level 2 khoảng 1/2 hành trình rồi thả ra.</t>
+  </si>
+  <si>
+    <t>1. Quạt đang chạy Mức 1.2. Dùng ngón tay ấn nhẹ nút Mức 2 khoảng 50% hành trình rồi nhả tay.</t>
+  </si>
+  <si>
+    <t>Nút Mức 1 vẫn giữ nguyên chốt (quạt tiếp tục chạy Mức 1), nút Mức 2 tự nảy về vị trí cũ nếu chưa đủ lực sập ngàm.</t>
+  </si>
+  <si>
+    <t>Nút Mức 1 bị nhả chốt làm quạt tắt hẳn, nhưng nút Mức 2 chưa đủ lực gài ngàm nên cũng nảy ra (quạt bị tắt nhầm).</t>
+  </si>
+  <si>
+    <t>FAIL (Kẹt chốt dở chừng)</t>
+  </si>
+  <si>
+    <t>TC16</t>
+  </si>
+  <si>
+    <t>TC17</t>
+  </si>
+  <si>
+    <t>TC18</t>
   </si>
 </sst>
 </file>
@@ -360,7 +426,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -383,39 +449,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -430,35 +468,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -1159,82 +1168,130 @@
       <c r="H16" s="4"/>
     </row>
     <row r="17" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="9"/>
+      <c r="H17" s="4"/>
     </row>
     <row r="18" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="G18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H18" s="16"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="11"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="11"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="11"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" ht="109.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="78" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>107</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>